<commit_message>
Score five unranked grants; sync spreadsheet with JSON
Adds estimates for the five foundation opportunities that had been
described in prose but never scored, bringing the ranked list to 23
scored plus 4 verify-first. Moves the Comer syringe services grant to
screened-out, since the org does not operate that service line.

Spreadsheet rank is now computed by sorting on win probability rather
than hardcoded, so adding a row or revising a score cannot desynchronise
the two files again. Both now hold 27 entries.
</commit_message>
<xml_diff>
--- a/grant_search/data/grant_pipeline.xlsx
+++ b/grant_search/data/grant_pipeline.xlsx
@@ -12,7 +12,7 @@
     <sheet name="Method" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Pipeline'!$A$4:$Q$26</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Pipeline'!$A$4:$Q$31</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -605,7 +605,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q30"/>
+  <dimension ref="A1:Q35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -1535,25 +1535,25 @@
       </c>
       <c r="B18" s="8" t="inlineStr">
         <is>
-          <t>Job Opportunities for Building Success</t>
+          <t>Therapeutic Giving: Neuroscience - Local &amp; Regional</t>
         </is>
       </c>
       <c r="C18" s="8" t="inlineStr">
         <is>
-          <t>NJ Dept. of Labor &amp; Workforce Dev.</t>
+          <t>Johnson &amp; Johnson Innovative Medicine</t>
         </is>
       </c>
       <c r="D18" s="9" t="inlineStr">
         <is>
-          <t>State / regional</t>
+          <t>Private foundation</t>
         </is>
       </c>
       <c r="E18" s="15" t="n">
-        <v>46450</v>
+        <v>46538</v>
       </c>
       <c r="F18" s="7" t="inlineStr">
         <is>
-          <t>LOI</t>
+          <t>Full</t>
         </is>
       </c>
       <c r="G18" s="7">
@@ -1561,15 +1561,13 @@
         <v/>
       </c>
       <c r="H18" s="10" t="n"/>
-      <c r="I18" s="10" t="n">
-        <v>1000000</v>
-      </c>
+      <c r="I18" s="10" t="n"/>
       <c r="J18" s="11">
         <f>IF(AND(H18&lt;&gt;"",I18&lt;&gt;""),AVERAGE(H18:I18),IF(I18&lt;&gt;"",I18*$C$3,IF(H18&lt;&gt;"",H18,"")))</f>
         <v/>
       </c>
       <c r="K18" s="12" t="n">
-        <v>0.1</v>
+        <v>0.12</v>
       </c>
       <c r="L18" s="11">
         <f>IF(OR(J18="",K18=""),"",J18*K18)</f>
@@ -1585,7 +1583,7 @@
       <c r="P18" s="14" t="n"/>
       <c r="Q18" s="8" t="inlineStr">
         <is>
-          <t>Reentry employment framing works, but competitors are established workforce development agencies.</t>
+          <t>Corporate giving with a local/regional track; mental health sits under its neuroscience umbrella. Pharma giving tends to favor established orgs and clinically-adjacent work, which caps the odds. Amount unpublished.</t>
         </is>
       </c>
     </row>
@@ -1595,21 +1593,21 @@
       </c>
       <c r="B19" s="8" t="inlineStr">
         <is>
-          <t>Second Chance Act - Family-Based SUD Treatment</t>
+          <t>Citizens Philanthropic Foundation: Workforce Development</t>
         </is>
       </c>
       <c r="C19" s="8" t="inlineStr">
         <is>
-          <t>US DOJ, BJA</t>
+          <t>Citizens Philanthropic Foundation</t>
         </is>
       </c>
       <c r="D19" s="9" t="inlineStr">
         <is>
-          <t>Federal</t>
+          <t>Private foundation</t>
         </is>
       </c>
       <c r="E19" s="15" t="n">
-        <v>46289</v>
+        <v>46529</v>
       </c>
       <c r="F19" s="7" t="inlineStr">
         <is>
@@ -1621,23 +1619,21 @@
         <v/>
       </c>
       <c r="H19" s="10" t="n"/>
-      <c r="I19" s="10" t="n">
-        <v>1000000</v>
-      </c>
+      <c r="I19" s="10" t="n"/>
       <c r="J19" s="11">
         <f>IF(AND(H19&lt;&gt;"",I19&lt;&gt;""),AVERAGE(H19:I19),IF(I19&lt;&gt;"",I19*$C$3,IF(H19&lt;&gt;"",H19,"")))</f>
         <v/>
       </c>
       <c r="K19" s="12" t="n">
-        <v>0.06</v>
+        <v>0.12</v>
       </c>
       <c r="L19" s="11">
         <f>IF(OR(J19="",K19=""),"",J19*K19)</f>
         <v/>
       </c>
-      <c r="M19" s="18" t="inlineStr">
-        <is>
-          <t>D</t>
+      <c r="M19" s="17" t="inlineStr">
+        <is>
+          <t>C</t>
         </is>
       </c>
       <c r="N19" s="14" t="n"/>
@@ -1645,7 +1641,7 @@
       <c r="P19" s="14" t="n"/>
       <c r="Q19" s="8" t="inlineStr">
         <is>
-          <t>BEST MISSION FIT on the entire list. Barriers: national competition, 3x-budget award, and the 'treatment provider' question (org refers out to IOP rather than treating directly). Pursue as partner/sub-awardee.</t>
+          <t>Reentry employment is a workable framing. Note this is the same corporate family as Champions in Action - a relationship built through one may help the other. Amount unpublished.</t>
         </is>
       </c>
     </row>
@@ -1655,25 +1651,25 @@
       </c>
       <c r="B20" s="8" t="inlineStr">
         <is>
-          <t>Second Chance Act - Reentry Education &amp; Employment</t>
+          <t>Job Opportunities for Building Success</t>
         </is>
       </c>
       <c r="C20" s="8" t="inlineStr">
         <is>
-          <t>US DOJ, BJA</t>
+          <t>NJ Dept. of Labor &amp; Workforce Dev.</t>
         </is>
       </c>
       <c r="D20" s="9" t="inlineStr">
         <is>
-          <t>Federal</t>
+          <t>State / regional</t>
         </is>
       </c>
       <c r="E20" s="15" t="n">
-        <v>46289</v>
+        <v>46450</v>
       </c>
       <c r="F20" s="7" t="inlineStr">
         <is>
-          <t>Full</t>
+          <t>LOI</t>
         </is>
       </c>
       <c r="G20" s="7">
@@ -1689,15 +1685,15 @@
         <v/>
       </c>
       <c r="K20" s="12" t="n">
-        <v>0.05</v>
+        <v>0.1</v>
       </c>
       <c r="L20" s="11">
         <f>IF(OR(J20="",K20=""),"",J20*K20)</f>
         <v/>
       </c>
-      <c r="M20" s="18" t="inlineStr">
-        <is>
-          <t>D</t>
+      <c r="M20" s="17" t="inlineStr">
+        <is>
+          <t>C</t>
         </is>
       </c>
       <c r="N20" s="14" t="n"/>
@@ -1705,7 +1701,7 @@
       <c r="P20" s="14" t="n"/>
       <c r="Q20" s="8" t="inlineStr">
         <is>
-          <t>Federal reentry competitions draw established national providers with prior DOJ awards. Pursue as partner/sub-awardee.</t>
+          <t>Reentry employment framing works, but competitors are established workforce development agencies.</t>
         </is>
       </c>
     </row>
@@ -1715,25 +1711,23 @@
       </c>
       <c r="B21" s="8" t="inlineStr">
         <is>
-          <t>Project Grant</t>
+          <t>Family foundations (Scripps, Kim/Kayasa, Bernau, Scaife)</t>
         </is>
       </c>
       <c r="C21" s="8" t="inlineStr">
         <is>
-          <t>State Justice Institute</t>
+          <t>Various</t>
         </is>
       </c>
       <c r="D21" s="9" t="inlineStr">
         <is>
-          <t>Federal</t>
-        </is>
-      </c>
-      <c r="E21" s="15" t="n">
-        <v>46327</v>
-      </c>
+          <t>Private foundation</t>
+        </is>
+      </c>
+      <c r="E21" s="7" t="n"/>
       <c r="F21" s="7" t="inlineStr">
         <is>
-          <t>Full</t>
+          <t>Rolling / 2027</t>
         </is>
       </c>
       <c r="G21" s="7">
@@ -1741,15 +1735,13 @@
         <v/>
       </c>
       <c r="H21" s="10" t="n"/>
-      <c r="I21" s="10" t="n">
-        <v>300000</v>
-      </c>
+      <c r="I21" s="10" t="n"/>
       <c r="J21" s="11">
         <f>IF(AND(H21&lt;&gt;"",I21&lt;&gt;""),AVERAGE(H21:I21),IF(I21&lt;&gt;"",I21*$C$3,IF(H21&lt;&gt;"",H21,"")))</f>
         <v/>
       </c>
       <c r="K21" s="12" t="n">
-        <v>0.05</v>
+        <v>0.1</v>
       </c>
       <c r="L21" s="11">
         <f>IF(OR(J21="",K21=""),"",J21*K21)</f>
@@ -1765,7 +1757,7 @@
       <c r="P21" s="14" t="n"/>
       <c r="Q21" s="8" t="inlineStr">
         <is>
-          <t>SJI funds court systems. Realistic path is as named program partner on a court-led application - the recovery court relationship could support that.</t>
+          <t>Priorities unpublished; many small family foundations are effectively invitation-only. Pull Form 990s before writing - 15 min each tells you whether they accept unsolicited requests at all.</t>
         </is>
       </c>
     </row>
@@ -1775,12 +1767,12 @@
       </c>
       <c r="B22" s="8" t="inlineStr">
         <is>
-          <t>Family foundations (Scripps, Kim/Kayasa, Bernau, Scaife)</t>
+          <t>Get Out and Get Active Grant</t>
         </is>
       </c>
       <c r="C22" s="8" t="inlineStr">
         <is>
-          <t>Various</t>
+          <t>Anxiety &amp; Depression Initiative</t>
         </is>
       </c>
       <c r="D22" s="9" t="inlineStr">
@@ -1788,10 +1780,12 @@
           <t>Private foundation</t>
         </is>
       </c>
-      <c r="E22" s="7" t="n"/>
+      <c r="E22" s="15" t="n">
+        <v>46504</v>
+      </c>
       <c r="F22" s="7" t="inlineStr">
         <is>
-          <t>Rolling / 2027</t>
+          <t>Full</t>
         </is>
       </c>
       <c r="G22" s="7">
@@ -1799,7 +1793,9 @@
         <v/>
       </c>
       <c r="H22" s="10" t="n"/>
-      <c r="I22" s="10" t="n"/>
+      <c r="I22" s="10" t="n">
+        <v>10000</v>
+      </c>
       <c r="J22" s="11">
         <f>IF(AND(H22&lt;&gt;"",I22&lt;&gt;""),AVERAGE(H22:I22),IF(I22&lt;&gt;"",I22*$C$3,IF(H22&lt;&gt;"",H22,"")))</f>
         <v/>
@@ -1811,9 +1807,9 @@
         <f>IF(OR(J22="",K22=""),"",J22*K22)</f>
         <v/>
       </c>
-      <c r="M22" s="18" t="inlineStr">
-        <is>
-          <t>D</t>
+      <c r="M22" s="17" t="inlineStr">
+        <is>
+          <t>C</t>
         </is>
       </c>
       <c r="N22" s="14" t="n"/>
@@ -1821,7 +1817,7 @@
       <c r="P22" s="14" t="n"/>
       <c r="Q22" s="8" t="inlineStr">
         <is>
-          <t>Priorities unpublished; many small family foundations are effectively invitation-only. Pull Form 990s before writing - 15 min each tells you whether they accept unsolicited requests at all.</t>
+          <t>PARTIAL FIT: this funder targets physical activity as an intervention for anxiety and depression. The org does psychoeducation and emotional wellness, not movement programming - a competitive application would need a genuine activity-based component, not a relabelling of existing workshops.</t>
         </is>
       </c>
     </row>
@@ -1831,21 +1827,21 @@
       </c>
       <c r="B23" s="8" t="inlineStr">
         <is>
-          <t>SNAP STEPS</t>
+          <t>JAMS Foundation NAFCM Mini-Grant Program</t>
         </is>
       </c>
       <c r="C23" s="8" t="inlineStr">
         <is>
-          <t>NJ Dept. of Labor &amp; Workforce Dev.</t>
+          <t>JAMS Foundation</t>
         </is>
       </c>
       <c r="D23" s="9" t="inlineStr">
         <is>
-          <t>State / regional</t>
+          <t>Private foundation</t>
         </is>
       </c>
       <c r="E23" s="15" t="n">
-        <v>46277</v>
+        <v>46441</v>
       </c>
       <c r="F23" s="7" t="inlineStr">
         <is>
@@ -1858,20 +1854,22 @@
       </c>
       <c r="H23" s="10" t="n"/>
       <c r="I23" s="10" t="n">
-        <v>500000</v>
+        <v>15000</v>
       </c>
       <c r="J23" s="11">
         <f>IF(AND(H23&lt;&gt;"",I23&lt;&gt;""),AVERAGE(H23:I23),IF(I23&lt;&gt;"",I23*$C$3,IF(H23&lt;&gt;"",H23,"")))</f>
         <v/>
       </c>
-      <c r="K23" s="12" t="n"/>
+      <c r="K23" s="12" t="n">
+        <v>0.08</v>
+      </c>
       <c r="L23" s="11">
         <f>IF(OR(J23="",K23=""),"",J23*K23)</f>
         <v/>
       </c>
-      <c r="M23" s="19" t="inlineStr">
-        <is>
-          <t>E</t>
+      <c r="M23" s="18" t="inlineStr">
+        <is>
+          <t>D</t>
         </is>
       </c>
       <c r="N23" s="14" t="n"/>
@@ -1879,7 +1877,7 @@
       <c r="P23" s="14" t="n"/>
       <c r="Q23" s="8" t="inlineStr">
         <is>
-          <t>VERIFY FIRST: near-term LOI. Overlap with reentry population is real but the org would need a workforce services track record.</t>
+          <t>ELIGIBILITY RISK: administered with the National Association for Community Mediation and generally aimed at NAFCM member community mediation centers. The org is not a mediation center. Anger management and healthy communication workshops map to the subject matter, but confirm whether non-member organizations can apply at all before spending time here.</t>
         </is>
       </c>
     </row>
@@ -1889,25 +1887,25 @@
       </c>
       <c r="B24" s="8" t="inlineStr">
         <is>
-          <t>Preventive Health Services Grant Program</t>
+          <t>Citizens Philanthropic Foundation: Financial Empowerment</t>
         </is>
       </c>
       <c r="C24" s="8" t="inlineStr">
         <is>
-          <t>NJ Dept. of Health</t>
+          <t>Citizens Philanthropic Foundation</t>
         </is>
       </c>
       <c r="D24" s="9" t="inlineStr">
         <is>
-          <t>State / regional</t>
+          <t>Private foundation</t>
         </is>
       </c>
       <c r="E24" s="15" t="n">
-        <v>46343</v>
+        <v>46357</v>
       </c>
       <c r="F24" s="7" t="inlineStr">
         <is>
-          <t>Full</t>
+          <t>Pre-proposal</t>
         </is>
       </c>
       <c r="G24" s="7">
@@ -1915,21 +1913,21 @@
         <v/>
       </c>
       <c r="H24" s="10" t="n"/>
-      <c r="I24" s="10" t="n">
-        <v>535000</v>
-      </c>
+      <c r="I24" s="10" t="n"/>
       <c r="J24" s="11">
         <f>IF(AND(H24&lt;&gt;"",I24&lt;&gt;""),AVERAGE(H24:I24),IF(I24&lt;&gt;"",I24*$C$3,IF(H24&lt;&gt;"",H24,"")))</f>
         <v/>
       </c>
-      <c r="K24" s="12" t="n"/>
+      <c r="K24" s="12" t="n">
+        <v>0.08</v>
+      </c>
       <c r="L24" s="11">
         <f>IF(OR(J24="",K24=""),"",J24*K24)</f>
         <v/>
       </c>
-      <c r="M24" s="19" t="inlineStr">
-        <is>
-          <t>E</t>
+      <c r="M24" s="18" t="inlineStr">
+        <is>
+          <t>D</t>
         </is>
       </c>
       <c r="N24" s="14" t="n"/>
@@ -1937,7 +1935,7 @@
       <c r="P24" s="14" t="n"/>
       <c r="Q24" s="8" t="inlineStr">
         <is>
-          <t>VERIFY FIRST: confirm community nonprofits are eligible applicants rather than local health departments.</t>
+          <t>Weakest fit of the five: this track funds financial literacy and coaching, which the org does not currently deliver. Nearest deadline of the group, but would require standing up a service line rather than describing one.</t>
         </is>
       </c>
     </row>
@@ -1947,21 +1945,21 @@
       </c>
       <c r="B25" s="8" t="inlineStr">
         <is>
-          <t>Omnibus Eviction and Homelessness Prevention</t>
+          <t>Second Chance Act - Family-Based SUD Treatment</t>
         </is>
       </c>
       <c r="C25" s="8" t="inlineStr">
         <is>
-          <t>NJ Dept. of Community Affairs</t>
+          <t>US DOJ, BJA</t>
         </is>
       </c>
       <c r="D25" s="9" t="inlineStr">
         <is>
-          <t>State / regional</t>
+          <t>Federal</t>
         </is>
       </c>
       <c r="E25" s="15" t="n">
-        <v>46358</v>
+        <v>46289</v>
       </c>
       <c r="F25" s="7" t="inlineStr">
         <is>
@@ -1973,19 +1971,23 @@
         <v/>
       </c>
       <c r="H25" s="10" t="n"/>
-      <c r="I25" s="10" t="n"/>
+      <c r="I25" s="10" t="n">
+        <v>1000000</v>
+      </c>
       <c r="J25" s="11">
         <f>IF(AND(H25&lt;&gt;"",I25&lt;&gt;""),AVERAGE(H25:I25),IF(I25&lt;&gt;"",I25*$C$3,IF(H25&lt;&gt;"",H25,"")))</f>
         <v/>
       </c>
-      <c r="K25" s="12" t="n"/>
+      <c r="K25" s="12" t="n">
+        <v>0.06</v>
+      </c>
       <c r="L25" s="11">
         <f>IF(OR(J25="",K25=""),"",J25*K25)</f>
         <v/>
       </c>
-      <c r="M25" s="19" t="inlineStr">
-        <is>
-          <t>E</t>
+      <c r="M25" s="18" t="inlineStr">
+        <is>
+          <t>D</t>
         </is>
       </c>
       <c r="N25" s="14" t="n"/>
@@ -1993,7 +1995,7 @@
       <c r="P25" s="14" t="n"/>
       <c r="Q25" s="8" t="inlineStr">
         <is>
-          <t>VERIFY FIRST: housing stability is adjacent to reentry wraparound; founder's lived experience with homelessness is relevant framing. Second RFP 2026-12-09.</t>
+          <t>BEST MISSION FIT on the entire list. Barriers: national competition, 3x-budget award, and the 'treatment provider' question (org refers out to IOP rather than treating directly). Pursue as partner/sub-awardee.</t>
         </is>
       </c>
     </row>
@@ -2003,25 +2005,25 @@
       </c>
       <c r="B26" s="8" t="inlineStr">
         <is>
-          <t>Chronic Disease Prevention Grant</t>
+          <t>Second Chance Act - Reentry Education &amp; Employment</t>
         </is>
       </c>
       <c r="C26" s="8" t="inlineStr">
         <is>
-          <t>NJ Dept. of Health</t>
+          <t>US DOJ, BJA</t>
         </is>
       </c>
       <c r="D26" s="9" t="inlineStr">
         <is>
-          <t>State / regional</t>
+          <t>Federal</t>
         </is>
       </c>
       <c r="E26" s="15" t="n">
-        <v>46379</v>
+        <v>46289</v>
       </c>
       <c r="F26" s="7" t="inlineStr">
         <is>
-          <t>LOI</t>
+          <t>Full</t>
         </is>
       </c>
       <c r="G26" s="7">
@@ -2030,20 +2032,22 @@
       </c>
       <c r="H26" s="10" t="n"/>
       <c r="I26" s="10" t="n">
-        <v>150000</v>
+        <v>1000000</v>
       </c>
       <c r="J26" s="11">
         <f>IF(AND(H26&lt;&gt;"",I26&lt;&gt;""),AVERAGE(H26:I26),IF(I26&lt;&gt;"",I26*$C$3,IF(H26&lt;&gt;"",H26,"")))</f>
         <v/>
       </c>
-      <c r="K26" s="12" t="n"/>
+      <c r="K26" s="12" t="n">
+        <v>0.05</v>
+      </c>
       <c r="L26" s="11">
         <f>IF(OR(J26="",K26=""),"",J26*K26)</f>
         <v/>
       </c>
-      <c r="M26" s="19" t="inlineStr">
-        <is>
-          <t>E</t>
+      <c r="M26" s="18" t="inlineStr">
+        <is>
+          <t>D</t>
         </is>
       </c>
       <c r="N26" s="14" t="n"/>
@@ -2051,45 +2055,335 @@
       <c r="P26" s="14" t="n"/>
       <c r="Q26" s="8" t="inlineStr">
         <is>
+          <t>Federal reentry competitions draw established national providers with prior DOJ awards. Pursue as partner/sub-awardee.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="46" customHeight="1">
+      <c r="A27" s="7" t="n">
+        <v>23</v>
+      </c>
+      <c r="B27" s="8" t="inlineStr">
+        <is>
+          <t>Project Grant</t>
+        </is>
+      </c>
+      <c r="C27" s="8" t="inlineStr">
+        <is>
+          <t>State Justice Institute</t>
+        </is>
+      </c>
+      <c r="D27" s="9" t="inlineStr">
+        <is>
+          <t>Federal</t>
+        </is>
+      </c>
+      <c r="E27" s="15" t="n">
+        <v>46327</v>
+      </c>
+      <c r="F27" s="7" t="inlineStr">
+        <is>
+          <t>Full</t>
+        </is>
+      </c>
+      <c r="G27" s="7">
+        <f>IF(E27="","",E27-TODAY())</f>
+        <v/>
+      </c>
+      <c r="H27" s="10" t="n"/>
+      <c r="I27" s="10" t="n">
+        <v>300000</v>
+      </c>
+      <c r="J27" s="11">
+        <f>IF(AND(H27&lt;&gt;"",I27&lt;&gt;""),AVERAGE(H27:I27),IF(I27&lt;&gt;"",I27*$C$3,IF(H27&lt;&gt;"",H27,"")))</f>
+        <v/>
+      </c>
+      <c r="K27" s="12" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="L27" s="11">
+        <f>IF(OR(J27="",K27=""),"",J27*K27)</f>
+        <v/>
+      </c>
+      <c r="M27" s="18" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="N27" s="14" t="n"/>
+      <c r="O27" s="14" t="n"/>
+      <c r="P27" s="14" t="n"/>
+      <c r="Q27" s="8" t="inlineStr">
+        <is>
+          <t>SJI funds court systems. Realistic path is as named program partner on a court-led application - the recovery court relationship could support that.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="46" customHeight="1">
+      <c r="A28" s="7" t="n">
+        <v>24</v>
+      </c>
+      <c r="B28" s="8" t="inlineStr">
+        <is>
+          <t>SNAP STEPS</t>
+        </is>
+      </c>
+      <c r="C28" s="8" t="inlineStr">
+        <is>
+          <t>NJ Dept. of Labor &amp; Workforce Dev.</t>
+        </is>
+      </c>
+      <c r="D28" s="9" t="inlineStr">
+        <is>
+          <t>State / regional</t>
+        </is>
+      </c>
+      <c r="E28" s="15" t="n">
+        <v>46277</v>
+      </c>
+      <c r="F28" s="7" t="inlineStr">
+        <is>
+          <t>LOI</t>
+        </is>
+      </c>
+      <c r="G28" s="7">
+        <f>IF(E28="","",E28-TODAY())</f>
+        <v/>
+      </c>
+      <c r="H28" s="10" t="n"/>
+      <c r="I28" s="10" t="n">
+        <v>500000</v>
+      </c>
+      <c r="J28" s="11">
+        <f>IF(AND(H28&lt;&gt;"",I28&lt;&gt;""),AVERAGE(H28:I28),IF(I28&lt;&gt;"",I28*$C$3,IF(H28&lt;&gt;"",H28,"")))</f>
+        <v/>
+      </c>
+      <c r="K28" s="12" t="n"/>
+      <c r="L28" s="11">
+        <f>IF(OR(J28="",K28=""),"",J28*K28)</f>
+        <v/>
+      </c>
+      <c r="M28" s="19" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+      <c r="N28" s="14" t="n"/>
+      <c r="O28" s="14" t="n"/>
+      <c r="P28" s="14" t="n"/>
+      <c r="Q28" s="8" t="inlineStr">
+        <is>
+          <t>VERIFY FIRST: near-term LOI. Overlap with reentry population is real but the org would need a workforce services track record.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="46" customHeight="1">
+      <c r="A29" s="7" t="n">
+        <v>25</v>
+      </c>
+      <c r="B29" s="8" t="inlineStr">
+        <is>
+          <t>Preventive Health Services Grant Program</t>
+        </is>
+      </c>
+      <c r="C29" s="8" t="inlineStr">
+        <is>
+          <t>NJ Dept. of Health</t>
+        </is>
+      </c>
+      <c r="D29" s="9" t="inlineStr">
+        <is>
+          <t>State / regional</t>
+        </is>
+      </c>
+      <c r="E29" s="15" t="n">
+        <v>46343</v>
+      </c>
+      <c r="F29" s="7" t="inlineStr">
+        <is>
+          <t>Full</t>
+        </is>
+      </c>
+      <c r="G29" s="7">
+        <f>IF(E29="","",E29-TODAY())</f>
+        <v/>
+      </c>
+      <c r="H29" s="10" t="n"/>
+      <c r="I29" s="10" t="n">
+        <v>535000</v>
+      </c>
+      <c r="J29" s="11">
+        <f>IF(AND(H29&lt;&gt;"",I29&lt;&gt;""),AVERAGE(H29:I29),IF(I29&lt;&gt;"",I29*$C$3,IF(H29&lt;&gt;"",H29,"")))</f>
+        <v/>
+      </c>
+      <c r="K29" s="12" t="n"/>
+      <c r="L29" s="11">
+        <f>IF(OR(J29="",K29=""),"",J29*K29)</f>
+        <v/>
+      </c>
+      <c r="M29" s="19" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+      <c r="N29" s="14" t="n"/>
+      <c r="O29" s="14" t="n"/>
+      <c r="P29" s="14" t="n"/>
+      <c r="Q29" s="8" t="inlineStr">
+        <is>
+          <t>VERIFY FIRST: confirm community nonprofits are eligible applicants rather than local health departments.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="46" customHeight="1">
+      <c r="A30" s="7" t="n">
+        <v>26</v>
+      </c>
+      <c r="B30" s="8" t="inlineStr">
+        <is>
+          <t>Omnibus Eviction and Homelessness Prevention</t>
+        </is>
+      </c>
+      <c r="C30" s="8" t="inlineStr">
+        <is>
+          <t>NJ Dept. of Community Affairs</t>
+        </is>
+      </c>
+      <c r="D30" s="9" t="inlineStr">
+        <is>
+          <t>State / regional</t>
+        </is>
+      </c>
+      <c r="E30" s="15" t="n">
+        <v>46358</v>
+      </c>
+      <c r="F30" s="7" t="inlineStr">
+        <is>
+          <t>Full</t>
+        </is>
+      </c>
+      <c r="G30" s="7">
+        <f>IF(E30="","",E30-TODAY())</f>
+        <v/>
+      </c>
+      <c r="H30" s="10" t="n"/>
+      <c r="I30" s="10" t="n"/>
+      <c r="J30" s="11">
+        <f>IF(AND(H30&lt;&gt;"",I30&lt;&gt;""),AVERAGE(H30:I30),IF(I30&lt;&gt;"",I30*$C$3,IF(H30&lt;&gt;"",H30,"")))</f>
+        <v/>
+      </c>
+      <c r="K30" s="12" t="n"/>
+      <c r="L30" s="11">
+        <f>IF(OR(J30="",K30=""),"",J30*K30)</f>
+        <v/>
+      </c>
+      <c r="M30" s="19" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+      <c r="N30" s="14" t="n"/>
+      <c r="O30" s="14" t="n"/>
+      <c r="P30" s="14" t="n"/>
+      <c r="Q30" s="8" t="inlineStr">
+        <is>
+          <t>VERIFY FIRST: housing stability is adjacent to reentry wraparound; founder's lived experience with homelessness is relevant framing. Second RFP 2026-12-09.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="46" customHeight="1">
+      <c r="A31" s="7" t="n">
+        <v>27</v>
+      </c>
+      <c r="B31" s="8" t="inlineStr">
+        <is>
+          <t>Chronic Disease Prevention Grant</t>
+        </is>
+      </c>
+      <c r="C31" s="8" t="inlineStr">
+        <is>
+          <t>NJ Dept. of Health</t>
+        </is>
+      </c>
+      <c r="D31" s="9" t="inlineStr">
+        <is>
+          <t>State / regional</t>
+        </is>
+      </c>
+      <c r="E31" s="15" t="n">
+        <v>46379</v>
+      </c>
+      <c r="F31" s="7" t="inlineStr">
+        <is>
+          <t>LOI</t>
+        </is>
+      </c>
+      <c r="G31" s="7">
+        <f>IF(E31="","",E31-TODAY())</f>
+        <v/>
+      </c>
+      <c r="H31" s="10" t="n"/>
+      <c r="I31" s="10" t="n">
+        <v>150000</v>
+      </c>
+      <c r="J31" s="11">
+        <f>IF(AND(H31&lt;&gt;"",I31&lt;&gt;""),AVERAGE(H31:I31),IF(I31&lt;&gt;"",I31*$C$3,IF(H31&lt;&gt;"",H31,"")))</f>
+        <v/>
+      </c>
+      <c r="K31" s="12" t="n"/>
+      <c r="L31" s="11">
+        <f>IF(OR(J31="",K31=""),"",J31*K31)</f>
+        <v/>
+      </c>
+      <c r="M31" s="19" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+      <c r="N31" s="14" t="n"/>
+      <c r="O31" s="14" t="n"/>
+      <c r="P31" s="14" t="n"/>
+      <c r="Q31" s="8" t="inlineStr">
+        <is>
           <t>VERIFY FIRST: often targeted at diabetes/cardiovascular - confirm behavioral health is in scope this cycle.</t>
         </is>
       </c>
     </row>
-    <row r="28">
-      <c r="B28" s="20" t="inlineStr">
+    <row r="33">
+      <c r="B33" s="20" t="inlineStr">
         <is>
           <t>TOTAL PIPELINE</t>
         </is>
       </c>
-      <c r="J28" s="21">
-        <f>SUM(J5:J26)</f>
-        <v/>
-      </c>
-      <c r="L28" s="21">
-        <f>SUM(L5:L26)</f>
-        <v/>
-      </c>
-      <c r="M28" s="5" t="inlineStr">
+      <c r="J33" s="21">
+        <f>SUM(J5:J31)</f>
+        <v/>
+      </c>
+      <c r="L33" s="21">
+        <f>SUM(L5:L31)</f>
+        <v/>
+      </c>
+      <c r="M33" s="5" t="inlineStr">
         <is>
           <t>&lt;- risk-weighted</t>
         </is>
       </c>
     </row>
-    <row r="30" ht="28" customHeight="1">
-      <c r="B30" s="2" t="inlineStr">
+    <row r="35" ht="28" customHeight="1">
+      <c r="B35" s="2" t="inlineStr">
         <is>
           <t>Expected Value = Planning Amount x Est. Win %. It is the risk-weighted worth of pursuing an item, NOT a forecast of what you will receive. Sorting by it gives a different order than sorting by likelihood - both are worth looking at.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:Q26"/>
+  <autoFilter ref="A4:Q31"/>
   <mergeCells count="2">
     <mergeCell ref="A2:Q2"/>
-    <mergeCell ref="B30:Q30"/>
+    <mergeCell ref="B35:Q35"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation sqref="N5:N26" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="N5:N31" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Not started,Researching,Drafting,Submitted,Awarded,Declined,Skipped"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Grant run 2026-08-23: Champions in Action upgraded to 18%
Confirms Citizens' budget eligibility band ($250k-$5M, so the org
qualifies), a broad and favourable 2026 theme, and an award that includes
volunteer engagement and promotion. Raises the estimate from 12% to 18%
and moves it into tier B.

Records the non-obvious catch: applicants must host 1-2 volunteer
projects for Citizens staff, at least one skills-based - an operational
commitment complicated by client confidentiality.

Also confirms behavioral health is the majority of HFNJ's non-hospital
grantmaking, strengthening that programmatic fit.
</commit_message>
<xml_diff>
--- a/grant_search/data/grant_pipeline.xlsx
+++ b/grant_search/data/grant_pipeline.xlsx
@@ -1293,49 +1293,51 @@
       </c>
       <c r="B14" s="8" t="inlineStr">
         <is>
-          <t>Pathways to Recovery - Round 2 NGO</t>
+          <t>Champions in Action</t>
         </is>
       </c>
       <c r="C14" s="8" t="inlineStr">
         <is>
-          <t>NJ Dept. of Labor &amp; Workforce Dev.</t>
+          <t>Citizens Charitable Foundation</t>
         </is>
       </c>
       <c r="D14" s="9" t="inlineStr">
         <is>
-          <t>State / regional</t>
+          <t>Private foundation</t>
         </is>
       </c>
       <c r="E14" s="15" t="n">
-        <v>46472</v>
+        <v>46295</v>
       </c>
       <c r="F14" s="7" t="inlineStr">
         <is>
-          <t>LOI</t>
+          <t>Full</t>
         </is>
       </c>
       <c r="G14" s="7">
         <f>IF(E14="","",E14-TODAY())</f>
         <v/>
       </c>
-      <c r="H14" s="10" t="n"/>
+      <c r="H14" s="10" t="n">
+        <v>50000</v>
+      </c>
       <c r="I14" s="10" t="n">
-        <v>1000000</v>
+        <v>50000</v>
       </c>
       <c r="J14" s="11">
         <f>IF(AND(H14&lt;&gt;"",I14&lt;&gt;""),AVERAGE(H14:I14),IF(I14&lt;&gt;"",I14*$C$3,IF(H14&lt;&gt;"",H14,"")))</f>
         <v/>
       </c>
       <c r="K14" s="12" t="n">
-        <v>0.15</v>
+        <v>0.18</v>
       </c>
       <c r="L14" s="11">
         <f>IF(OR(J14="",K14=""),"",J14*K14)</f>
         <v/>
       </c>
-      <c r="M14" s="17" t="inlineStr">
-        <is>
-          <t>C</t>
+      <c r="M14" s="16" t="inlineStr">
+        <is>
+          <t>B</t>
         </is>
       </c>
       <c r="N14" s="14" t="n"/>
@@ -1343,7 +1345,7 @@
       <c r="P14" s="14" t="n"/>
       <c r="Q14" s="8" t="inlineStr">
         <is>
-          <t>HIGHEST EXPECTED VALUE on the list. NJ-only pool, NGO-specific track, opioid focus matches directly. Ask well under the cap.</t>
+          <t>UPGRADED 2026-08-23. Budget eligibility confirmed ($250k-$5M; the org qualifies). 2026 theme 'Uplifting Resilient Nonprofits' is broad and favourable. Award is $50k plus volunteer engagement and promotion. CATCH: applicants must host 1-2 volunteer projects for Citizens staff, at least one skills-based - needs a credible plan given client confidentiality.</t>
         </is>
       </c>
     </row>
@@ -1353,7 +1355,7 @@
       </c>
       <c r="B15" s="8" t="inlineStr">
         <is>
-          <t>Pathways to Recovery (general)</t>
+          <t>Pathways to Recovery - Round 2 NGO</t>
         </is>
       </c>
       <c r="C15" s="8" t="inlineStr">
@@ -1367,7 +1369,7 @@
         </is>
       </c>
       <c r="E15" s="15" t="n">
-        <v>46451</v>
+        <v>46472</v>
       </c>
       <c r="F15" s="7" t="inlineStr">
         <is>
@@ -1387,7 +1389,7 @@
         <v/>
       </c>
       <c r="K15" s="12" t="n">
-        <v>0.12</v>
+        <v>0.15</v>
       </c>
       <c r="L15" s="11">
         <f>IF(OR(J15="",K15=""),"",J15*K15)</f>
@@ -1403,7 +1405,7 @@
       <c r="P15" s="14" t="n"/>
       <c r="Q15" s="8" t="inlineStr">
         <is>
-          <t>Same program, broader applicant pool than the NGO track.</t>
+          <t>HIGHEST EXPECTED VALUE on the list. NJ-only pool, NGO-specific track, opioid focus matches directly. Ask well under the cap.</t>
         </is>
       </c>
     </row>
@@ -1413,36 +1415,34 @@
       </c>
       <c r="B16" s="8" t="inlineStr">
         <is>
-          <t>Champions in Action</t>
+          <t>Pathways to Recovery (general)</t>
         </is>
       </c>
       <c r="C16" s="8" t="inlineStr">
         <is>
-          <t>Citizens Charitable Foundation</t>
+          <t>NJ Dept. of Labor &amp; Workforce Dev.</t>
         </is>
       </c>
       <c r="D16" s="9" t="inlineStr">
         <is>
-          <t>Private foundation</t>
+          <t>State / regional</t>
         </is>
       </c>
       <c r="E16" s="15" t="n">
-        <v>46295</v>
+        <v>46451</v>
       </c>
       <c r="F16" s="7" t="inlineStr">
         <is>
-          <t>Full</t>
+          <t>LOI</t>
         </is>
       </c>
       <c r="G16" s="7">
         <f>IF(E16="","",E16-TODAY())</f>
         <v/>
       </c>
-      <c r="H16" s="10" t="n">
-        <v>50000</v>
-      </c>
+      <c r="H16" s="10" t="n"/>
       <c r="I16" s="10" t="n">
-        <v>50000</v>
+        <v>1000000</v>
       </c>
       <c r="J16" s="11">
         <f>IF(AND(H16&lt;&gt;"",I16&lt;&gt;""),AVERAGE(H16:I16),IF(I16&lt;&gt;"",I16*$C$3,IF(H16&lt;&gt;"",H16,"")))</f>
@@ -1465,7 +1465,7 @@
       <c r="P16" s="14" t="n"/>
       <c r="Q16" s="8" t="inlineStr">
         <is>
-          <t>Selects very few recipients per cycle, usually themed. Check this round's theme.</t>
+          <t>Same program, broader applicant pool than the NGO track.</t>
         </is>
       </c>
     </row>

</xml_diff>